<commit_message>
Deploying to gh-pages from @ yugandharreddy0718/smartstudyai@d0d275136eb63a236d7dd2adc768a7ecdcb29133 🚀
</commit_message>
<xml_diff>
--- a/reports/Mobile/appium-report.xlsx
+++ b/reports/Mobile/appium-report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="120">
   <si>
     <t>SMARTSTUDY AI - ANDROID APPIUM E2E TEST REPORT</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>18.59 seconds</t>
+    <t>18.60 seconds</t>
   </si>
   <si>
     <t>Execution Platform</t>
@@ -56,7 +56,7 @@
     <t>Date &amp; Time</t>
   </si>
   <si>
-    <t>8/27/2026, 4:40:05 PM</t>
+    <t>10/8/2026, 3:15:59 PM</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -98,10 +98,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:46.812Z</t>
-  </si>
-  <si>
-    <t>2026-08-27T16:39:48.014Z</t>
+    <t>2026-10-08T15:15:41.336Z</t>
+  </si>
+  <si>
+    <t>2026-10-08T15:15:42.538Z</t>
   </si>
   <si>
     <t>Verified successfully.</t>
@@ -116,7 +116,7 @@
     <t>Mobile Login Screen &amp; Form Rendering</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:48.615Z</t>
+    <t>2026-10-08T15:15:43.139Z</t>
   </si>
   <si>
     <t>APP-003</t>
@@ -125,7 +125,7 @@
     <t>Invalid Mobile Login Error Handling</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:49.216Z</t>
+    <t>2026-10-08T15:15:43.741Z</t>
   </si>
   <si>
     <t>APP-004</t>
@@ -137,10 +137,7 @@
     <t>Student Dashboard &amp; Subject Grid Cards</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:49.217Z</t>
-  </si>
-  <si>
-    <t>2026-08-27T16:39:49.819Z</t>
+    <t>2026-10-08T15:15:44.342Z</t>
   </si>
   <si>
     <t>APP-005</t>
@@ -152,7 +149,7 @@
     <t>Switch Active Grade to Class 6</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:50.420Z</t>
+    <t>2026-10-08T15:15:44.943Z</t>
   </si>
   <si>
     <t>APP-006</t>
@@ -161,7 +158,7 @@
     <t>Switch Active Grade to Class 7</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:51.021Z</t>
+    <t>2026-10-08T15:15:45.544Z</t>
   </si>
   <si>
     <t>APP-007</t>
@@ -170,7 +167,7 @@
     <t>Switch Active Grade to Class 8</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:51.622Z</t>
+    <t>2026-10-08T15:15:46.145Z</t>
   </si>
   <si>
     <t>APP-008</t>
@@ -179,7 +176,7 @@
     <t>Switch Active Grade to Class 9</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:52.223Z</t>
+    <t>2026-10-08T15:15:46.746Z</t>
   </si>
   <si>
     <t>APP-009</t>
@@ -188,7 +185,7 @@
     <t>Switch Active Grade to Class 10</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:52.825Z</t>
+    <t>2026-10-08T15:15:47.347Z</t>
   </si>
   <si>
     <t>APP-010</t>
@@ -200,7 +197,7 @@
     <t>Explore Mathematics Stream Grid</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:53.425Z</t>
+    <t>2026-10-08T15:15:47.948Z</t>
   </si>
   <si>
     <t>APP-011</t>
@@ -209,10 +206,7 @@
     <t>Explore Physics, Chemistry &amp; Biology Streams</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:53.426Z</t>
-  </si>
-  <si>
-    <t>2026-08-27T16:39:54.026Z</t>
+    <t>2026-10-08T15:15:48.549Z</t>
   </si>
   <si>
     <t>APP-012</t>
@@ -221,7 +215,7 @@
     <t>Explore History, Civics &amp; Geography Streams</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:54.628Z</t>
+    <t>2026-10-08T15:15:49.150Z</t>
   </si>
   <si>
     <t>APP-013</t>
@@ -233,7 +227,7 @@
     <t>Chapter Catalog Navigation &amp; Sub-lesson Catalog</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:55.228Z</t>
+    <t>2026-10-08T15:15:49.751Z</t>
   </si>
   <si>
     <t>APP-014</t>
@@ -245,7 +239,7 @@
     <t>Verify 13-Section Pedagogical Layout Rendering</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:57.030Z</t>
+    <t>2026-10-08T15:15:51.553Z</t>
   </si>
   <si>
     <t>APP-015</t>
@@ -257,7 +251,7 @@
     <t>Trigger Mark Lesson Complete &amp; XP Award (+100 XP)</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:57.631Z</t>
+    <t>2026-10-08T15:15:52.154Z</t>
   </si>
   <si>
     <t>APP-016</t>
@@ -269,7 +263,7 @@
     <t>AI Studio — Interactive Summary Tool</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:58.233Z</t>
+    <t>2026-10-08T15:15:52.755Z</t>
   </si>
   <si>
     <t>APP-017</t>
@@ -281,7 +275,7 @@
     <t>AI Studio — High-Yield Exam Q&amp;A Generator</t>
   </si>
   <si>
-    <t>2026-08-27T16:39:58.834Z</t>
+    <t>2026-10-08T15:15:53.356Z</t>
   </si>
   <si>
     <t>APP-018</t>
@@ -293,7 +287,7 @@
     <t>AI Studio — Standalone MCQ Generator</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:00.836Z</t>
+    <t>2026-10-08T15:15:55.358Z</t>
   </si>
   <si>
     <t>APP-019</t>
@@ -305,7 +299,7 @@
     <t>AI Studio — Interactive Quiz Assessment</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:01.437Z</t>
+    <t>2026-10-08T15:15:55.959Z</t>
   </si>
   <si>
     <t>APP-020</t>
@@ -317,7 +311,7 @@
     <t>AI Studio — 24/7 AI Tutor Chat Assistant Interface</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:02.038Z</t>
+    <t>2026-10-08T15:15:56.560Z</t>
   </si>
   <si>
     <t>APP-021</t>
@@ -329,7 +323,7 @@
     <t>Mobile Document Upload &amp; OCR Text Extraction Studio</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:02.639Z</t>
+    <t>2026-10-08T15:15:57.161Z</t>
   </si>
   <si>
     <t>APP-022</t>
@@ -341,7 +335,7 @@
     <t>Mobile PDF Reader &amp; Document Viewer Tools</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:03.240Z</t>
+    <t>2026-10-08T15:15:57.762Z</t>
   </si>
   <si>
     <t>APP-023</t>
@@ -353,7 +347,7 @@
     <t>Execute Search Query across Curriculum Index</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:03.841Z</t>
+    <t>2026-10-08T15:15:58.363Z</t>
   </si>
   <si>
     <t>APP-024</t>
@@ -365,7 +359,7 @@
     <t>Student Profile Stats &amp; Session Logout Execution</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:04.442Z</t>
+    <t>2026-10-08T15:15:58.964Z</t>
   </si>
   <si>
     <t>APP-025</t>
@@ -377,7 +371,7 @@
     <t>Protected Route Access Control &amp; Security Check</t>
   </si>
   <si>
-    <t>2026-08-27T16:40:05.043Z</t>
+    <t>2026-10-08T15:15:59.565Z</t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1004,7 @@
         <v>27</v>
       </c>
       <c r="E4">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F4" t="s">
         <v>34</v>
@@ -1039,13 +1033,13 @@
         <v>27</v>
       </c>
       <c r="E5">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
         <v>41</v>
-      </c>
-      <c r="G5" t="s">
-        <v>42</v>
       </c>
       <c r="H5" t="s">
         <v>30</v>
@@ -1056,25 +1050,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
         <v>43</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>44</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>601</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
         <v>45</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6">
-        <v>601</v>
-      </c>
-      <c r="F6" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" t="s">
-        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>30</v>
@@ -1085,25 +1079,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7">
+        <v>601</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
         <v>48</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7">
-        <v>601</v>
-      </c>
-      <c r="F7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
       </c>
       <c r="H7" t="s">
         <v>30</v>
@@ -1114,25 +1108,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
         <v>50</v>
       </c>
-      <c r="B8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <v>601</v>
+      </c>
+      <c r="F8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" t="s">
         <v>51</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>601</v>
-      </c>
-      <c r="F8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" t="s">
-        <v>52</v>
       </c>
       <c r="H8" t="s">
         <v>30</v>
@@ -1143,25 +1137,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9">
+        <v>601</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
         <v>54</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9">
-        <v>601</v>
-      </c>
-      <c r="F9" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" t="s">
-        <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>30</v>
@@ -1172,25 +1166,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
         <v>56</v>
       </c>
-      <c r="B10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10">
+        <v>601</v>
+      </c>
+      <c r="F10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" t="s">
         <v>57</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10">
-        <v>602</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" t="s">
-        <v>58</v>
       </c>
       <c r="H10" t="s">
         <v>30</v>
@@ -1201,25 +1195,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
         <v>59</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>60</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11">
+        <v>601</v>
+      </c>
+      <c r="F11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" t="s">
         <v>61</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11">
-        <v>601</v>
-      </c>
-      <c r="F11" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" t="s">
-        <v>62</v>
       </c>
       <c r="H11" t="s">
         <v>30</v>
@@ -1230,25 +1224,25 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" t="s">
         <v>63</v>
       </c>
-      <c r="B12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>601</v>
+      </c>
+      <c r="F12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" t="s">
         <v>64</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12">
-        <v>600</v>
-      </c>
-      <c r="F12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" t="s">
-        <v>66</v>
       </c>
       <c r="H12" t="s">
         <v>30</v>
@@ -1259,25 +1253,25 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13">
+        <v>601</v>
+      </c>
+      <c r="F13" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" t="s">
         <v>67</v>
-      </c>
-      <c r="B13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13">
-        <v>602</v>
-      </c>
-      <c r="F13" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13" t="s">
-        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>30</v>
@@ -1288,25 +1282,25 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
         <v>70</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14">
+        <v>601</v>
+      </c>
+      <c r="F14" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" t="s">
         <v>71</v>
-      </c>
-      <c r="C14" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14">
-        <v>600</v>
-      </c>
-      <c r="F14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" t="s">
-        <v>73</v>
       </c>
       <c r="H14" t="s">
         <v>30</v>
@@ -1317,13 +1311,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" t="s">
         <v>74</v>
-      </c>
-      <c r="B15" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" t="s">
-        <v>76</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>27</v>
@@ -1332,10 +1326,10 @@
         <v>1802</v>
       </c>
       <c r="F15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H15" t="s">
         <v>30</v>
@@ -1346,25 +1340,25 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" t="s">
         <v>78</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16">
+        <v>601</v>
+      </c>
+      <c r="F16" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" t="s">
         <v>79</v>
-      </c>
-      <c r="C16" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16">
-        <v>601</v>
-      </c>
-      <c r="F16" t="s">
-        <v>77</v>
-      </c>
-      <c r="G16" t="s">
-        <v>81</v>
       </c>
       <c r="H16" t="s">
         <v>30</v>
@@ -1375,25 +1369,25 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" t="s">
         <v>82</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17">
+        <v>601</v>
+      </c>
+      <c r="F17" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" t="s">
         <v>83</v>
-      </c>
-      <c r="C17" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17">
-        <v>602</v>
-      </c>
-      <c r="F17" t="s">
-        <v>81</v>
-      </c>
-      <c r="G17" t="s">
-        <v>85</v>
       </c>
       <c r="H17" t="s">
         <v>30</v>
@@ -1404,25 +1398,25 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" t="s">
         <v>86</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18">
+        <v>601</v>
+      </c>
+      <c r="F18" t="s">
+        <v>83</v>
+      </c>
+      <c r="G18" t="s">
         <v>87</v>
-      </c>
-      <c r="C18" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18">
-        <v>601</v>
-      </c>
-      <c r="F18" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" t="s">
-        <v>89</v>
       </c>
       <c r="H18" t="s">
         <v>30</v>
@@ -1433,13 +1427,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" t="s">
         <v>90</v>
-      </c>
-      <c r="B19" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" t="s">
-        <v>92</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>27</v>
@@ -1448,10 +1442,10 @@
         <v>2002</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H19" t="s">
         <v>30</v>
@@ -1462,25 +1456,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" t="s">
+        <v>93</v>
+      </c>
+      <c r="C20" t="s">
         <v>94</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20">
+        <v>601</v>
+      </c>
+      <c r="F20" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" t="s">
         <v>95</v>
-      </c>
-      <c r="C20" t="s">
-        <v>96</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20">
-        <v>601</v>
-      </c>
-      <c r="F20" t="s">
-        <v>93</v>
-      </c>
-      <c r="G20" t="s">
-        <v>97</v>
       </c>
       <c r="H20" t="s">
         <v>30</v>
@@ -1491,25 +1485,25 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" t="s">
         <v>98</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21">
+        <v>601</v>
+      </c>
+      <c r="F21" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" t="s">
         <v>99</v>
-      </c>
-      <c r="C21" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21">
-        <v>601</v>
-      </c>
-      <c r="F21" t="s">
-        <v>97</v>
-      </c>
-      <c r="G21" t="s">
-        <v>101</v>
       </c>
       <c r="H21" t="s">
         <v>30</v>
@@ -1520,25 +1514,25 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" t="s">
         <v>102</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22">
+        <v>601</v>
+      </c>
+      <c r="F22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22" t="s">
         <v>103</v>
-      </c>
-      <c r="C22" t="s">
-        <v>104</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22">
-        <v>601</v>
-      </c>
-      <c r="F22" t="s">
-        <v>101</v>
-      </c>
-      <c r="G22" t="s">
-        <v>105</v>
       </c>
       <c r="H22" t="s">
         <v>30</v>
@@ -1549,25 +1543,25 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" t="s">
         <v>106</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23">
+        <v>601</v>
+      </c>
+      <c r="F23" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" t="s">
         <v>107</v>
-      </c>
-      <c r="C23" t="s">
-        <v>108</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23">
-        <v>601</v>
-      </c>
-      <c r="F23" t="s">
-        <v>105</v>
-      </c>
-      <c r="G23" t="s">
-        <v>109</v>
       </c>
       <c r="H23" t="s">
         <v>30</v>
@@ -1578,25 +1572,25 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" t="s">
         <v>110</v>
       </c>
-      <c r="B24" t="s">
+      <c r="D24" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24">
+        <v>601</v>
+      </c>
+      <c r="F24" t="s">
+        <v>107</v>
+      </c>
+      <c r="G24" t="s">
         <v>111</v>
-      </c>
-      <c r="C24" t="s">
-        <v>112</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24">
-        <v>601</v>
-      </c>
-      <c r="F24" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" t="s">
-        <v>113</v>
       </c>
       <c r="H24" t="s">
         <v>30</v>
@@ -1607,25 +1601,25 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25" t="s">
         <v>114</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25">
+        <v>601</v>
+      </c>
+      <c r="F25" t="s">
+        <v>111</v>
+      </c>
+      <c r="G25" t="s">
         <v>115</v>
-      </c>
-      <c r="C25" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25">
-        <v>601</v>
-      </c>
-      <c r="F25" t="s">
-        <v>113</v>
-      </c>
-      <c r="G25" t="s">
-        <v>117</v>
       </c>
       <c r="H25" t="s">
         <v>30</v>
@@ -1636,25 +1630,25 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" t="s">
+        <v>117</v>
+      </c>
+      <c r="C26" t="s">
         <v>118</v>
       </c>
-      <c r="B26" t="s">
+      <c r="D26" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26">
+        <v>601</v>
+      </c>
+      <c r="F26" t="s">
+        <v>115</v>
+      </c>
+      <c r="G26" t="s">
         <v>119</v>
-      </c>
-      <c r="C26" t="s">
-        <v>120</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26">
-        <v>601</v>
-      </c>
-      <c r="F26" t="s">
-        <v>117</v>
-      </c>
-      <c r="G26" t="s">
-        <v>121</v>
       </c>
       <c r="H26" t="s">
         <v>30</v>

</xml_diff>